<commit_message>
Update permissions for AE2 and AE3 Excel files
</commit_message>
<xml_diff>
--- a/docs/Ae2.xlsx
+++ b/docs/Ae2.xlsx
@@ -479,12 +479,12 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>MES: 5 2026</t>
+          <t>MES: 12 2024</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>FECHA:11-5-2026</t>
+          <t>FECHA:1-12-2024</t>
         </is>
       </c>
     </row>
@@ -526,15 +526,11 @@
           <t>1.- Total Plantilla Aprobada</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
-      <c r="F11" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -542,15 +538,11 @@
           <t>2.- Total Plantilla Cubierta</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
-        <v>1732</v>
-      </c>
+      <c r="B12" s="5" t="n"/>
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
-      <c r="F12" s="6" t="n">
-        <v>1732</v>
-      </c>
+      <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -558,15 +550,11 @@
           <t>3.- Total General de Contratos</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
-        <v>2348</v>
-      </c>
+      <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n">
-        <v>2348</v>
-      </c>
+      <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -574,15 +562,11 @@
           <t>4.- Total de Contratos de Profesores por tiempo determinado</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B14" s="5" t="n"/>
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="5" t="n"/>
-      <c r="F14" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -590,15 +574,11 @@
           <t>5.- De ellos: a tiempo completo</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="n"/>
-      <c r="F15" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -606,15 +586,11 @@
           <t>6.- Total de Contratos No Docentes</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
-        <v>2348</v>
-      </c>
+      <c r="B16" s="6" t="n"/>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n">
-        <v>2348</v>
-      </c>
+      <c r="F16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -622,15 +598,11 @@
           <t>7.- Contratos No Docentes con respaldo de plazas</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
-        <v>2348</v>
-      </c>
+      <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n">
-        <v>2348</v>
-      </c>
+      <c r="F17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -638,15 +610,11 @@
           <t>8.- De ellos: por sustitución</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="B18" s="5" t="n"/>
       <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
-      <c r="F18" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="F18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -654,15 +622,11 @@
           <t>9.- Período de Prueba</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
-        <v>68</v>
-      </c>
+      <c r="B19" s="5" t="n"/>
       <c r="C19" s="5" t="n"/>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
-      <c r="F19" s="6" t="n">
-        <v>68</v>
-      </c>
+      <c r="F19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -670,15 +634,11 @@
           <t>10.- Serenos y Auxiliares de Limpieza</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
-        <v>108</v>
-      </c>
+      <c r="B20" s="5" t="n"/>
       <c r="C20" s="5" t="n"/>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
-      <c r="F20" s="6" t="n">
-        <v>108</v>
-      </c>
+      <c r="F20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -686,15 +646,11 @@
           <t>11.- Labores Agrícolas</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B21" s="5" t="n"/>
       <c r="C21" s="5" t="n"/>
       <c r="D21" s="5" t="n"/>
       <c r="E21" s="5" t="n"/>
-      <c r="F21" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -702,15 +658,11 @@
           <t>12.- Jubilados</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
-        <v>105</v>
-      </c>
+      <c r="B22" s="5" t="n"/>
       <c r="C22" s="5" t="n"/>
       <c r="D22" s="5" t="n"/>
       <c r="E22" s="5" t="n"/>
-      <c r="F22" s="6" t="n">
-        <v>105</v>
-      </c>
+      <c r="F22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -718,15 +670,11 @@
           <t>13.- Otros</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B23" s="5" t="n"/>
       <c r="C23" s="5" t="n"/>
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="5" t="n"/>
-      <c r="F23" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -734,15 +682,11 @@
           <t>14.- Contratos No Docentes sin respaldo de plazas (15 a 19)</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="B24" s="6" t="n"/>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
       <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -750,15 +694,11 @@
           <t>15.- De ellos: Serenos y Auxiliares de Limpieza</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B25" s="5" t="n"/>
       <c r="C25" s="5" t="n"/>
       <c r="D25" s="5" t="n"/>
       <c r="E25" s="5" t="n"/>
-      <c r="F25" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -766,15 +706,11 @@
           <t>16.- Ejecución de Obra</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B26" s="5" t="n"/>
       <c r="C26" s="5" t="n"/>
       <c r="D26" s="5" t="n"/>
       <c r="E26" s="5" t="n"/>
-      <c r="F26" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -782,15 +718,11 @@
           <t>17.- Reserva Científica en Preparación</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B27" s="5" t="n"/>
       <c r="C27" s="5" t="n"/>
       <c r="D27" s="5" t="n"/>
       <c r="E27" s="5" t="n"/>
-      <c r="F27" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -798,15 +730,11 @@
           <t>18.- Recién Graduados en Preparación</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B28" s="5" t="n"/>
       <c r="C28" s="5" t="n"/>
       <c r="D28" s="5" t="n"/>
       <c r="E28" s="5" t="n"/>
-      <c r="F28" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -814,15 +742,11 @@
           <t>19.- Reserva Dirección Provincial de Trabajo</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
-        <v>311</v>
-      </c>
+      <c r="B29" s="5" t="n"/>
       <c r="C29" s="5" t="n"/>
       <c r="D29" s="5" t="n"/>
       <c r="E29" s="5" t="n"/>
-      <c r="F29" s="6" t="n">
-        <v>311</v>
-      </c>
+      <c r="F29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -830,15 +754,11 @@
           <t>20.- Técnicos Medios en Preparación</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B30" s="5" t="n"/>
       <c r="C30" s="5" t="n"/>
       <c r="D30" s="5" t="n"/>
       <c r="E30" s="5" t="n"/>
-      <c r="F30" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -846,15 +766,11 @@
           <t>21 - Total de estudiantes de la Universidad de CD contratados por tiempo determinado</t>
         </is>
       </c>
-      <c r="B31" s="6" t="n">
-        <v>311</v>
-      </c>
+      <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n">
-        <v>311</v>
-      </c>
+      <c r="F31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -862,15 +778,11 @@
           <t>22 - Del total de estudiantes de CD contratados, cifras como Auxiliar Técnico de la Docencia</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B32" s="5" t="n"/>
       <c r="C32" s="5" t="n"/>
       <c r="D32" s="5" t="n"/>
       <c r="E32" s="5" t="n"/>
-      <c r="F32" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -878,15 +790,11 @@
           <t>23 - Del total de estudiantes de CD contratados, cifras en cargos No Docentes</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B33" s="5" t="n"/>
       <c r="C33" s="5" t="n"/>
       <c r="D33" s="5" t="n"/>
       <c r="E33" s="5" t="n"/>
-      <c r="F33" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="F33" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
@@ -898,14 +806,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Confeccionado por:    pepe                                     Revisado por:admin</t>
+          <t>Confeccionado por:    None                                     Revisado por:None</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">                           presorrrssss                                                               admin</t>
+          <t xml:space="preserve">                           None                                                               None</t>
         </is>
       </c>
     </row>

</xml_diff>